<commit_message>
Mise à jour hebdomadaire des données de cardiologie 🔄
</commit_message>
<xml_diff>
--- a/fhf_cardiologie.xlsx
+++ b/fhf_cardiologie.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>benedicte.point@ch-laon.fr</t>
+          <t>moudo.megherbi@ch-laon.fr</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>c.balluais@ch-compiegnenoyon.fr</t>
+          <t>e.deliancourt@ch-compiegnenoyon.fr</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">

</xml_diff>